<commit_message>
modify discriminator Practitioner.qualification 8a9055fc2f60a0bfbc405fd74112ec06a99d64b2
</commit_message>
<xml_diff>
--- a/110-creation-exemples/ig/StructureDefinition-as-dp-practitioner.xlsx
+++ b/110-creation-exemples/ig/StructureDefinition-as-dp-practitioner.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11058" uniqueCount="980">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11058" uniqueCount="979">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-02T11:51:09+00:00</t>
+    <t>2024-07-02T12:01:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2538,7 +2538,7 @@
     <t>The official certifications, training, and licenses that authorize or otherwise pertain to the provision of care by the practitioner.  For example, a medical license issued by a medical board authorizing the practitioner to practice medicine within a certian locality.</t>
   </si>
   <si>
-    <t xml:space="preserve">value:code}
+    <t xml:space="preserve">pattern:$this}
 </t>
   </si>
   <si>
@@ -2792,10 +2792,6 @@
   </si>
   <si>
     <t>Practitioner.qualification.code.coding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pattern:$this}
-</t>
   </si>
   <si>
     <t>Practitioner.qualification:degree.code.coding:degreeType</t>
@@ -32943,7 +32939,7 @@
         <v>78</v>
       </c>
       <c r="AB254" t="s" s="2">
-        <v>892</v>
+        <v>808</v>
       </c>
       <c r="AC254" s="2"/>
       <c r="AD254" t="s" s="2">
@@ -32985,13 +32981,13 @@
     </row>
     <row r="255" hidden="true">
       <c r="A255" t="s" s="2">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B255" t="s" s="2">
         <v>891</v>
       </c>
       <c r="C255" t="s" s="2">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="D255" t="s" s="2">
         <v>78</v>
@@ -33054,7 +33050,7 @@
       </c>
       <c r="Y255" s="2"/>
       <c r="Z255" t="s" s="2">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="AA255" t="s" s="2">
         <v>78</v>
@@ -33104,7 +33100,7 @@
     </row>
     <row r="256" hidden="true">
       <c r="A256" t="s" s="2">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B256" t="s" s="2">
         <v>891</v>
@@ -33223,10 +33219,10 @@
     </row>
     <row r="257" hidden="true">
       <c r="A257" t="s" s="2">
+        <v>896</v>
+      </c>
+      <c r="B257" t="s" s="2">
         <v>897</v>
-      </c>
-      <c r="B257" t="s" s="2">
-        <v>898</v>
       </c>
       <c r="C257" s="2"/>
       <c r="D257" t="s" s="2">
@@ -33342,7 +33338,7 @@
     </row>
     <row r="258" hidden="true">
       <c r="A258" t="s" s="2">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B258" t="s" s="2">
         <v>829</v>
@@ -33371,7 +33367,7 @@
         <v>253</v>
       </c>
       <c r="L258" t="s" s="2">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M258" t="s" s="2">
         <v>831</v>
@@ -33459,10 +33455,10 @@
     </row>
     <row r="259" hidden="true">
       <c r="A259" t="s" s="2">
+        <v>900</v>
+      </c>
+      <c r="B259" t="s" s="2">
         <v>901</v>
-      </c>
-      <c r="B259" t="s" s="2">
-        <v>902</v>
       </c>
       <c r="C259" s="2"/>
       <c r="D259" t="s" s="2">
@@ -33574,10 +33570,10 @@
     </row>
     <row r="260" hidden="true">
       <c r="A260" t="s" s="2">
+        <v>902</v>
+      </c>
+      <c r="B260" t="s" s="2">
         <v>903</v>
-      </c>
-      <c r="B260" t="s" s="2">
-        <v>904</v>
       </c>
       <c r="C260" s="2"/>
       <c r="D260" t="s" s="2">
@@ -33691,10 +33687,10 @@
     </row>
     <row r="261" hidden="true">
       <c r="A261" t="s" s="2">
+        <v>904</v>
+      </c>
+      <c r="B261" t="s" s="2">
         <v>905</v>
-      </c>
-      <c r="B261" t="s" s="2">
-        <v>906</v>
       </c>
       <c r="C261" s="2"/>
       <c r="D261" t="s" s="2">
@@ -33720,7 +33716,7 @@
         <v>260</v>
       </c>
       <c r="L261" t="s" s="2">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="M261" t="s" s="2">
         <v>262</v>
@@ -33808,10 +33804,10 @@
     </row>
     <row r="262" hidden="true">
       <c r="A262" t="s" s="2">
+        <v>907</v>
+      </c>
+      <c r="B262" t="s" s="2">
         <v>908</v>
-      </c>
-      <c r="B262" t="s" s="2">
-        <v>909</v>
       </c>
       <c r="C262" s="2"/>
       <c r="D262" t="s" s="2">
@@ -33837,7 +33833,7 @@
         <v>260</v>
       </c>
       <c r="L262" t="s" s="2">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="M262" t="s" s="2">
         <v>271</v>
@@ -33927,7 +33923,7 @@
     </row>
     <row r="263" hidden="true">
       <c r="A263" t="s" s="2">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B263" t="s" s="2">
         <v>835</v>
@@ -33953,10 +33949,10 @@
         <v>78</v>
       </c>
       <c r="K263" t="s" s="2">
+        <v>911</v>
+      </c>
+      <c r="L263" t="s" s="2">
         <v>912</v>
-      </c>
-      <c r="L263" t="s" s="2">
-        <v>913</v>
       </c>
       <c r="M263" t="s" s="2">
         <v>837</v>
@@ -34042,13 +34038,13 @@
     </row>
     <row r="264" hidden="true">
       <c r="A264" t="s" s="2">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B264" t="s" s="2">
         <v>804</v>
       </c>
       <c r="C264" t="s" s="2">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="D264" t="s" s="2">
         <v>78</v>
@@ -34073,7 +34069,7 @@
         <v>805</v>
       </c>
       <c r="L264" t="s" s="2">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="M264" t="s" s="2">
         <v>807</v>
@@ -34159,7 +34155,7 @@
     </row>
     <row r="265" hidden="true">
       <c r="A265" t="s" s="2">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="B265" t="s" s="2">
         <v>812</v>
@@ -34274,7 +34270,7 @@
     </row>
     <row r="266" hidden="true">
       <c r="A266" t="s" s="2">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B266" t="s" s="2">
         <v>813</v>
@@ -34391,7 +34387,7 @@
     </row>
     <row r="267" hidden="true">
       <c r="A267" t="s" s="2">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="B267" t="s" s="2">
         <v>814</v>
@@ -34510,7 +34506,7 @@
     </row>
     <row r="268" hidden="true">
       <c r="A268" t="s" s="2">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="B268" t="s" s="2">
         <v>819</v>
@@ -34627,7 +34623,7 @@
     </row>
     <row r="269" hidden="true">
       <c r="A269" t="s" s="2">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="B269" t="s" s="2">
         <v>824</v>
@@ -34740,7 +34736,7 @@
     </row>
     <row r="270" hidden="true">
       <c r="A270" t="s" s="2">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="B270" t="s" s="2">
         <v>887</v>
@@ -34855,7 +34851,7 @@
     </row>
     <row r="271" hidden="true">
       <c r="A271" t="s" s="2">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="B271" t="s" s="2">
         <v>889</v>
@@ -34972,7 +34968,7 @@
     </row>
     <row r="272" hidden="true">
       <c r="A272" t="s" s="2">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B272" t="s" s="2">
         <v>891</v>
@@ -35047,7 +35043,7 @@
         <v>78</v>
       </c>
       <c r="AB272" t="s" s="2">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="AC272" s="2"/>
       <c r="AD272" t="s" s="2">
@@ -35089,13 +35085,13 @@
     </row>
     <row r="273" hidden="true">
       <c r="A273" t="s" s="2">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B273" t="s" s="2">
         <v>891</v>
       </c>
       <c r="C273" t="s" s="2">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="D273" t="s" s="2">
         <v>78</v>
@@ -35120,7 +35116,7 @@
         <v>154</v>
       </c>
       <c r="L273" t="s" s="2">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="M273" t="s" s="2">
         <v>395</v>
@@ -35158,7 +35154,7 @@
       </c>
       <c r="Y273" s="2"/>
       <c r="Z273" t="s" s="2">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="AA273" t="s" s="2">
         <v>78</v>
@@ -35208,7 +35204,7 @@
     </row>
     <row r="274" hidden="true">
       <c r="A274" t="s" s="2">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B274" t="s" s="2">
         <v>891</v>
@@ -35239,7 +35235,7 @@
         <v>154</v>
       </c>
       <c r="L274" t="s" s="2">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="M274" t="s" s="2">
         <v>395</v>
@@ -35327,10 +35323,10 @@
     </row>
     <row r="275" hidden="true">
       <c r="A275" t="s" s="2">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B275" t="s" s="2">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C275" s="2"/>
       <c r="D275" t="s" s="2">
@@ -35446,7 +35442,7 @@
     </row>
     <row r="276" hidden="true">
       <c r="A276" t="s" s="2">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="B276" t="s" s="2">
         <v>829</v>
@@ -35563,10 +35559,10 @@
     </row>
     <row r="277" hidden="true">
       <c r="A277" t="s" s="2">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B277" t="s" s="2">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C277" s="2"/>
       <c r="D277" t="s" s="2">
@@ -35678,10 +35674,10 @@
     </row>
     <row r="278" hidden="true">
       <c r="A278" t="s" s="2">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B278" t="s" s="2">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C278" s="2"/>
       <c r="D278" t="s" s="2">
@@ -35795,10 +35791,10 @@
     </row>
     <row r="279" hidden="true">
       <c r="A279" t="s" s="2">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="B279" t="s" s="2">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="C279" s="2"/>
       <c r="D279" t="s" s="2">
@@ -35824,7 +35820,7 @@
         <v>260</v>
       </c>
       <c r="L279" t="s" s="2">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="M279" t="s" s="2">
         <v>262</v>
@@ -35912,10 +35908,10 @@
     </row>
     <row r="280" hidden="true">
       <c r="A280" t="s" s="2">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B280" t="s" s="2">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C280" s="2"/>
       <c r="D280" t="s" s="2">
@@ -35941,7 +35937,7 @@
         <v>260</v>
       </c>
       <c r="L280" t="s" s="2">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="M280" t="s" s="2">
         <v>271</v>
@@ -36031,7 +36027,7 @@
     </row>
     <row r="281" hidden="true">
       <c r="A281" t="s" s="2">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B281" t="s" s="2">
         <v>835</v>
@@ -36146,13 +36142,13 @@
     </row>
     <row r="282" hidden="true">
       <c r="A282" t="s" s="2">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="B282" t="s" s="2">
         <v>804</v>
       </c>
       <c r="C282" t="s" s="2">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="D282" t="s" s="2">
         <v>78</v>
@@ -36177,7 +36173,7 @@
         <v>805</v>
       </c>
       <c r="L282" t="s" s="2">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="M282" t="s" s="2">
         <v>807</v>
@@ -36263,7 +36259,7 @@
     </row>
     <row r="283" hidden="true">
       <c r="A283" t="s" s="2">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="B283" t="s" s="2">
         <v>812</v>
@@ -36378,7 +36374,7 @@
     </row>
     <row r="284" hidden="true">
       <c r="A284" t="s" s="2">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="B284" t="s" s="2">
         <v>813</v>
@@ -36495,7 +36491,7 @@
     </row>
     <row r="285" hidden="true">
       <c r="A285" t="s" s="2">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="B285" t="s" s="2">
         <v>814</v>
@@ -36614,7 +36610,7 @@
     </row>
     <row r="286" hidden="true">
       <c r="A286" t="s" s="2">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B286" t="s" s="2">
         <v>819</v>
@@ -36731,7 +36727,7 @@
     </row>
     <row r="287" hidden="true">
       <c r="A287" t="s" s="2">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B287" t="s" s="2">
         <v>824</v>
@@ -36827,7 +36823,7 @@
         <v>102</v>
       </c>
       <c r="AK287" t="s" s="2">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="AL287" t="s" s="2">
         <v>78</v>
@@ -36844,7 +36840,7 @@
     </row>
     <row r="288" hidden="true">
       <c r="A288" t="s" s="2">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B288" t="s" s="2">
         <v>887</v>
@@ -36959,7 +36955,7 @@
     </row>
     <row r="289" hidden="true">
       <c r="A289" t="s" s="2">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B289" t="s" s="2">
         <v>889</v>
@@ -37076,7 +37072,7 @@
     </row>
     <row r="290" hidden="true">
       <c r="A290" t="s" s="2">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B290" t="s" s="2">
         <v>891</v>
@@ -37151,7 +37147,7 @@
         <v>78</v>
       </c>
       <c r="AB290" t="s" s="2">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="AC290" s="2"/>
       <c r="AD290" t="s" s="2">
@@ -37193,13 +37189,13 @@
     </row>
     <row r="291" hidden="true">
       <c r="A291" t="s" s="2">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B291" t="s" s="2">
         <v>891</v>
       </c>
       <c r="C291" t="s" s="2">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D291" t="s" s="2">
         <v>78</v>
@@ -37224,7 +37220,7 @@
         <v>154</v>
       </c>
       <c r="L291" t="s" s="2">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="M291" t="s" s="2">
         <v>395</v>
@@ -37262,7 +37258,7 @@
       </c>
       <c r="Y291" s="2"/>
       <c r="Z291" t="s" s="2">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="AA291" t="s" s="2">
         <v>78</v>
@@ -37312,13 +37308,13 @@
     </row>
     <row r="292" hidden="true">
       <c r="A292" t="s" s="2">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="B292" t="s" s="2">
         <v>891</v>
       </c>
       <c r="C292" t="s" s="2">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="D292" t="s" s="2">
         <v>78</v>
@@ -37343,7 +37339,7 @@
         <v>154</v>
       </c>
       <c r="L292" t="s" s="2">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="M292" t="s" s="2">
         <v>395</v>
@@ -37381,7 +37377,7 @@
       </c>
       <c r="Y292" s="2"/>
       <c r="Z292" t="s" s="2">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="AA292" t="s" s="2">
         <v>78</v>
@@ -37431,10 +37427,10 @@
     </row>
     <row r="293" hidden="true">
       <c r="A293" t="s" s="2">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B293" t="s" s="2">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C293" s="2"/>
       <c r="D293" t="s" s="2">
@@ -37550,7 +37546,7 @@
     </row>
     <row r="294" hidden="true">
       <c r="A294" t="s" s="2">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B294" t="s" s="2">
         <v>829</v>
@@ -37667,10 +37663,10 @@
     </row>
     <row r="295" hidden="true">
       <c r="A295" t="s" s="2">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B295" t="s" s="2">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C295" s="2"/>
       <c r="D295" t="s" s="2">
@@ -37782,10 +37778,10 @@
     </row>
     <row r="296" hidden="true">
       <c r="A296" t="s" s="2">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B296" t="s" s="2">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C296" s="2"/>
       <c r="D296" t="s" s="2">
@@ -37899,10 +37895,10 @@
     </row>
     <row r="297" hidden="true">
       <c r="A297" t="s" s="2">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B297" t="s" s="2">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="C297" s="2"/>
       <c r="D297" t="s" s="2">
@@ -37928,7 +37924,7 @@
         <v>260</v>
       </c>
       <c r="L297" t="s" s="2">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="M297" t="s" s="2">
         <v>262</v>
@@ -37999,7 +37995,7 @@
         <v>102</v>
       </c>
       <c r="AK297" t="s" s="2">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="AL297" t="s" s="2">
         <v>266</v>
@@ -38016,10 +38012,10 @@
     </row>
     <row r="298" hidden="true">
       <c r="A298" t="s" s="2">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B298" t="s" s="2">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C298" s="2"/>
       <c r="D298" t="s" s="2">
@@ -38045,7 +38041,7 @@
         <v>260</v>
       </c>
       <c r="L298" t="s" s="2">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="M298" t="s" s="2">
         <v>271</v>
@@ -38118,7 +38114,7 @@
         <v>102</v>
       </c>
       <c r="AK298" t="s" s="2">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="AL298" t="s" s="2">
         <v>275</v>
@@ -38135,7 +38131,7 @@
     </row>
     <row r="299" hidden="true">
       <c r="A299" t="s" s="2">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B299" t="s" s="2">
         <v>835</v>
@@ -38250,10 +38246,10 @@
     </row>
     <row r="300" hidden="true">
       <c r="A300" t="s" s="2">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B300" t="s" s="2">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="C300" s="2"/>
       <c r="D300" t="s" s="2">
@@ -38276,19 +38272,19 @@
         <v>78</v>
       </c>
       <c r="K300" t="s" s="2">
+        <v>971</v>
+      </c>
+      <c r="L300" t="s" s="2">
         <v>972</v>
       </c>
-      <c r="L300" t="s" s="2">
+      <c r="M300" t="s" s="2">
         <v>973</v>
       </c>
-      <c r="M300" t="s" s="2">
+      <c r="N300" t="s" s="2">
         <v>974</v>
       </c>
-      <c r="N300" t="s" s="2">
+      <c r="O300" t="s" s="2">
         <v>975</v>
-      </c>
-      <c r="O300" t="s" s="2">
-        <v>976</v>
       </c>
       <c r="P300" t="s" s="2">
         <v>78</v>
@@ -38317,7 +38313,7 @@
       </c>
       <c r="Y300" s="2"/>
       <c r="Z300" t="s" s="2">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AA300" t="s" s="2">
         <v>78</v>
@@ -38335,7 +38331,7 @@
         <v>78</v>
       </c>
       <c r="AF300" t="s" s="2">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="AG300" t="s" s="2">
         <v>79</v>
@@ -38353,10 +38349,10 @@
         <v>78</v>
       </c>
       <c r="AL300" t="s" s="2">
+        <v>977</v>
+      </c>
+      <c r="AM300" t="s" s="2">
         <v>978</v>
-      </c>
-      <c r="AM300" t="s" s="2">
-        <v>979</v>
       </c>
       <c r="AN300" t="s" s="2">
         <v>78</v>

</xml_diff>